<commit_message>
Experimento 18 e atualização de documentação
</commit_message>
<xml_diff>
--- a/Project_CNN/Main/Results/Experimento 10 - ResNet/training_metrics.xlsx
+++ b/Project_CNN/Main/Results/Experimento 10 - ResNet/training_metrics.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marci_wawp\Desktop\Arquivos\Mestrado\Projeto-Classificadores\Main_Project\ResNet\Results\Experimento 10 -ResNet\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marci_wawp\Desktop\Arquivos\Mestrado\Projeto-Classificadores\Project_CNN\Main\Results\Experimento 10 - ResNet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5C83E42-51D3-4F34-AAA8-164A27F96E9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E689498-48A2-49C2-8E0C-4578F85585D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-21720" yWindow="2520" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worksheet" sheetId="1" r:id="rId1"/>

</xml_diff>